<commit_message>
feat: coisas novas ai
</commit_message>
<xml_diff>
--- a/produtos_classificados.xlsx
+++ b/produtos_classificados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\GitHub\cadastro_sku\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA6C8081-6473-410B-9226-14D95E4EC9CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5F93253-8B7F-456A-8FF7-927284D32BFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="1755" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="385">
   <si>
     <t>SKU</t>
   </si>
@@ -631,9 +631,6 @@
     <t>Relogio Redondo Dourado Menor 02</t>
   </si>
   <si>
-    <t>RELOGIO-REDONDO-PRATA-01</t>
-  </si>
-  <si>
     <t>Relogio Redondo Prata 01</t>
   </si>
   <si>
@@ -649,21 +646,12 @@
     <t>Relogio Redondo Menor Rose</t>
   </si>
   <si>
-    <t>RELOGIO-REDODNO-PRETO-01</t>
-  </si>
-  <si>
     <t>Relogio Redodno Preto 01</t>
   </si>
   <si>
-    <t>RELOGIO-REDONDO-PRETO-02</t>
-  </si>
-  <si>
     <t>Relogio Redondo Preto 02</t>
   </si>
   <si>
-    <t>RELOGIO-REDONDO-MAIOR-01</t>
-  </si>
-  <si>
     <t>Relogio Redondo Maior 01</t>
   </si>
   <si>
@@ -1172,14 +1160,37 @@
   </si>
   <si>
     <t>RELOGIO-MASCULINO-PRETO-AMARELO</t>
+  </si>
+  <si>
+    <t>RELOGIO-REDONDO-PRATA-MAIOR-01</t>
+  </si>
+  <si>
+    <t>RELOGIO-REDODNO-PRETO-MENOR-01</t>
+  </si>
+  <si>
+    <t>RELOGIO-REDONDO-PRETO-MENOR-02</t>
+  </si>
+  <si>
+    <t>RELOGIO-REDONDO-DOURADO-MAIOR-01</t>
+  </si>
+  <si>
+    <t>Cadastrado</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1207,8 +1218,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1511,16 +1523,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E179"/>
+  <dimension ref="A1:G179"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="79.42578125" customWidth="1"/>
     <col min="2" max="2" width="79.85546875" customWidth="1"/>
     <col min="3" max="3" width="24.5703125" customWidth="1"/>
     <col min="4" max="4" width="30.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1533,8 +1546,11 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1547,8 +1563,11 @@
       <c r="D2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1561,8 +1580,11 @@
       <c r="D3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1575,8 +1597,12 @@
       <c r="D4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1589,8 +1615,11 @@
       <c r="D5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1603,8 +1632,11 @@
       <c r="D6" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1617,8 +1649,11 @@
       <c r="D7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -1631,8 +1666,11 @@
       <c r="D8" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1646,7 +1684,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1659,8 +1697,11 @@
       <c r="D10" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -1673,8 +1714,11 @@
       <c r="D11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>26</v>
       </c>
@@ -1687,8 +1731,11 @@
       <c r="D12" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -1701,8 +1748,11 @@
       <c r="D13" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>30</v>
       </c>
@@ -1715,8 +1765,11 @@
       <c r="D14" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -1726,11 +1779,14 @@
       <c r="C15" t="s">
         <v>6</v>
       </c>
-      <c r="D15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D15" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>34</v>
       </c>
@@ -1742,6 +1798,9 @@
       </c>
       <c r="D16" t="s">
         <v>7</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1757,6 +1816,9 @@
       <c r="D17" t="s">
         <v>7</v>
       </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -1771,6 +1833,9 @@
       <c r="D18" t="s">
         <v>7</v>
       </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -1785,6 +1850,9 @@
       <c r="D19" t="s">
         <v>7</v>
       </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
@@ -1799,6 +1867,9 @@
       <c r="D20" t="s">
         <v>7</v>
       </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -1813,6 +1884,9 @@
       <c r="D21" t="s">
         <v>7</v>
       </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -1827,6 +1901,9 @@
       <c r="D22" t="s">
         <v>7</v>
       </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
@@ -1855,6 +1932,9 @@
       <c r="D24" t="s">
         <v>7</v>
       </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -1869,6 +1949,9 @@
       <c r="D25" t="s">
         <v>7</v>
       </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
@@ -1883,6 +1966,9 @@
       <c r="D26" t="s">
         <v>7</v>
       </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
@@ -1897,6 +1983,9 @@
       <c r="D27" t="s">
         <v>7</v>
       </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
@@ -1911,6 +2000,9 @@
       <c r="D28" t="s">
         <v>7</v>
       </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
@@ -1925,6 +2017,9 @@
       <c r="D29" t="s">
         <v>7</v>
       </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
@@ -1939,6 +2034,9 @@
       <c r="D30" t="s">
         <v>7</v>
       </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
@@ -1953,6 +2051,7 @@
       <c r="D31" t="s">
         <v>7</v>
       </c>
+      <c r="E31" s="1"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -2063,6 +2162,9 @@
       <c r="D38" t="s">
         <v>7</v>
       </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
@@ -2142,6 +2244,9 @@
       <c r="D43" t="s">
         <v>7</v>
       </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
@@ -2156,6 +2261,9 @@
       <c r="D44" t="s">
         <v>7</v>
       </c>
+      <c r="E44">
+        <v>1</v>
+      </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
@@ -2170,6 +2278,9 @@
       <c r="D45" t="s">
         <v>7</v>
       </c>
+      <c r="E45">
+        <v>1</v>
+      </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
@@ -2198,6 +2309,9 @@
       <c r="D47" t="s">
         <v>7</v>
       </c>
+      <c r="E47">
+        <v>1</v>
+      </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
@@ -2212,6 +2326,9 @@
       <c r="D48" t="s">
         <v>7</v>
       </c>
+      <c r="E48">
+        <v>1</v>
+      </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
@@ -2268,6 +2385,9 @@
       <c r="D52" t="s">
         <v>7</v>
       </c>
+      <c r="E52">
+        <v>1</v>
+      </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -2282,6 +2402,9 @@
       <c r="D53" t="s">
         <v>7</v>
       </c>
+      <c r="E53">
+        <v>1</v>
+      </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
@@ -2296,6 +2419,9 @@
       <c r="D54" t="s">
         <v>7</v>
       </c>
+      <c r="E54">
+        <v>1</v>
+      </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
@@ -2310,6 +2436,9 @@
       <c r="D55" t="s">
         <v>7</v>
       </c>
+      <c r="E55">
+        <v>1</v>
+      </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
@@ -2372,6 +2501,9 @@
       <c r="D59" t="s">
         <v>7</v>
       </c>
+      <c r="E59">
+        <v>1</v>
+      </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
@@ -2400,6 +2532,9 @@
       <c r="D61" t="s">
         <v>7</v>
       </c>
+      <c r="E61">
+        <v>1</v>
+      </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
@@ -2414,6 +2549,9 @@
       <c r="D62" t="s">
         <v>7</v>
       </c>
+      <c r="E62">
+        <v>1</v>
+      </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
@@ -2442,8 +2580,11 @@
       <c r="D64" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>132</v>
       </c>
@@ -2457,7 +2598,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>134</v>
       </c>
@@ -2471,7 +2612,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>136</v>
       </c>
@@ -2485,7 +2626,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>138</v>
       </c>
@@ -2499,7 +2640,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>140</v>
       </c>
@@ -2513,7 +2654,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>142</v>
       </c>
@@ -2527,7 +2668,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>144</v>
       </c>
@@ -2540,8 +2681,11 @@
       <c r="D71" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E71">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>146</v>
       </c>
@@ -2555,7 +2699,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>148</v>
       </c>
@@ -2569,7 +2713,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>150</v>
       </c>
@@ -2583,7 +2727,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>152</v>
       </c>
@@ -2597,7 +2741,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>154</v>
       </c>
@@ -2611,7 +2755,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>156</v>
       </c>
@@ -2625,7 +2769,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>158</v>
       </c>
@@ -2639,7 +2783,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>160</v>
       </c>
@@ -2652,8 +2796,11 @@
       <c r="D79" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E79">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>162</v>
       </c>
@@ -2665,6 +2812,9 @@
       </c>
       <c r="D80" t="s">
         <v>7</v>
+      </c>
+      <c r="E80">
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
@@ -2739,6 +2889,9 @@
       <c r="D85" t="s">
         <v>7</v>
       </c>
+      <c r="E85">
+        <v>1</v>
+      </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
@@ -2753,6 +2906,9 @@
       <c r="D86" t="s">
         <v>7</v>
       </c>
+      <c r="E86">
+        <v>1</v>
+      </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
@@ -2770,7 +2926,7 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="B88" t="s">
         <v>178</v>
@@ -2784,7 +2940,7 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="B89" t="s">
         <v>179</v>
@@ -2928,6 +3084,9 @@
       <c r="D97" t="s">
         <v>200</v>
       </c>
+      <c r="E97">
+        <v>1</v>
+      </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
@@ -2942,13 +3101,16 @@
       <c r="D98" t="s">
         <v>200</v>
       </c>
+      <c r="E98">
+        <v>1</v>
+      </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
+        <v>380</v>
+      </c>
+      <c r="B99" t="s">
         <v>203</v>
-      </c>
-      <c r="B99" t="s">
-        <v>204</v>
       </c>
       <c r="C99" t="s">
         <v>6</v>
@@ -2956,13 +3118,16 @@
       <c r="D99" t="s">
         <v>200</v>
       </c>
+      <c r="E99">
+        <v>1</v>
+      </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
+        <v>204</v>
+      </c>
+      <c r="B100" t="s">
         <v>205</v>
-      </c>
-      <c r="B100" t="s">
-        <v>206</v>
       </c>
       <c r="C100" t="s">
         <v>6</v>
@@ -2970,13 +3135,16 @@
       <c r="D100" t="s">
         <v>200</v>
       </c>
+      <c r="E100">
+        <v>1</v>
+      </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
+        <v>206</v>
+      </c>
+      <c r="B101" t="s">
         <v>207</v>
-      </c>
-      <c r="B101" t="s">
-        <v>208</v>
       </c>
       <c r="C101" t="s">
         <v>6</v>
@@ -2984,13 +3152,16 @@
       <c r="D101" t="s">
         <v>200</v>
       </c>
+      <c r="E101">
+        <v>1</v>
+      </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>209</v>
+        <v>381</v>
       </c>
       <c r="B102" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C102" t="s">
         <v>6</v>
@@ -2998,13 +3169,16 @@
       <c r="D102" t="s">
         <v>200</v>
       </c>
+      <c r="E102">
+        <v>1</v>
+      </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>211</v>
+        <v>382</v>
       </c>
       <c r="B103" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C103" t="s">
         <v>6</v>
@@ -3012,13 +3186,16 @@
       <c r="D103" t="s">
         <v>200</v>
       </c>
+      <c r="E103">
+        <v>1</v>
+      </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>213</v>
+        <v>383</v>
       </c>
       <c r="B104" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="C104" t="s">
         <v>6</v>
@@ -3026,13 +3203,16 @@
       <c r="D104" t="s">
         <v>200</v>
       </c>
+      <c r="E104">
+        <v>1</v>
+      </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="B105" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="C105" t="s">
         <v>6</v>
@@ -3040,13 +3220,16 @@
       <c r="D105" t="s">
         <v>200</v>
       </c>
+      <c r="E105">
+        <v>1</v>
+      </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="B106" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="C106" t="s">
         <v>6</v>
@@ -3054,13 +3237,16 @@
       <c r="D106" t="s">
         <v>200</v>
       </c>
+      <c r="E106">
+        <v>1</v>
+      </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="B107" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="C107" t="s">
         <v>6</v>
@@ -3068,13 +3254,16 @@
       <c r="D107" t="s">
         <v>200</v>
       </c>
+      <c r="E107">
+        <v>1</v>
+      </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="B108" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="C108" t="s">
         <v>6</v>
@@ -3082,13 +3271,16 @@
       <c r="D108" t="s">
         <v>200</v>
       </c>
+      <c r="E108">
+        <v>1</v>
+      </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="B109" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="C109" t="s">
         <v>6</v>
@@ -3096,13 +3288,16 @@
       <c r="D109" t="s">
         <v>200</v>
       </c>
+      <c r="E109">
+        <v>1</v>
+      </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B110" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="C110" t="s">
         <v>6</v>
@@ -3116,10 +3311,10 @@
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B111" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="C111" t="s">
         <v>6</v>
@@ -3133,10 +3328,10 @@
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B112" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="C112" t="s">
         <v>6</v>
@@ -3150,10 +3345,10 @@
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="B113" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="C113" t="s">
         <v>6</v>
@@ -3167,10 +3362,10 @@
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="B114" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="C114" t="s">
         <v>6</v>
@@ -3184,10 +3379,10 @@
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B115" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="C115" t="s">
         <v>6</v>
@@ -3201,10 +3396,10 @@
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="B116" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C116" t="s">
         <v>6</v>
@@ -3218,10 +3413,10 @@
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="B117" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="C117" t="s">
         <v>6</v>
@@ -3235,10 +3430,10 @@
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="B118" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="C118" t="s">
         <v>6</v>
@@ -3252,10 +3447,10 @@
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="B119" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="C119" t="s">
         <v>6</v>
@@ -3269,10 +3464,10 @@
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="B120" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="C120" t="s">
         <v>6</v>
@@ -3286,10 +3481,10 @@
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="B121" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="C121" t="s">
         <v>6</v>
@@ -3303,10 +3498,10 @@
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="B122" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="C122" t="s">
         <v>6</v>
@@ -3320,10 +3515,10 @@
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="B123" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="C123" t="s">
         <v>6</v>
@@ -3337,10 +3532,10 @@
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B124" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="C124" t="s">
         <v>6</v>
@@ -3354,10 +3549,10 @@
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="B125" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="C125" t="s">
         <v>6</v>
@@ -3365,13 +3560,16 @@
       <c r="D125" t="s">
         <v>200</v>
       </c>
+      <c r="E125">
+        <v>1</v>
+      </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="B126" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="C126" t="s">
         <v>6</v>
@@ -3379,13 +3577,16 @@
       <c r="D126" t="s">
         <v>200</v>
       </c>
+      <c r="E126">
+        <v>1</v>
+      </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="B127" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="C127" t="s">
         <v>6</v>
@@ -3399,10 +3600,10 @@
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="B128" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C128" t="s">
         <v>6</v>
@@ -3416,10 +3617,10 @@
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="B129" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="C129" t="s">
         <v>6</v>
@@ -3433,10 +3634,10 @@
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="B130" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="C130" t="s">
         <v>6</v>
@@ -3450,10 +3651,10 @@
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="B131" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="C131" t="s">
         <v>6</v>
@@ -3461,13 +3662,16 @@
       <c r="D131" t="s">
         <v>200</v>
       </c>
+      <c r="E131">
+        <v>1</v>
+      </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="B132" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="C132" t="s">
         <v>6</v>
@@ -3481,10 +3685,10 @@
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="B133" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="C133" t="s">
         <v>6</v>
@@ -3498,10 +3702,10 @@
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="B134" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="C134" t="s">
         <v>6</v>
@@ -3515,16 +3719,16 @@
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="B135" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="C135" t="s">
         <v>6</v>
       </c>
       <c r="D135" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -3532,16 +3736,16 @@
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="B136" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="C136" t="s">
         <v>6</v>
       </c>
       <c r="D136" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -3549,16 +3753,16 @@
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="B137" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="C137" t="s">
         <v>6</v>
       </c>
       <c r="D137" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -3566,16 +3770,16 @@
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="B138" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="C138" t="s">
         <v>6</v>
       </c>
       <c r="D138" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -3583,16 +3787,16 @@
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="B139" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="C139" t="s">
         <v>6</v>
       </c>
       <c r="D139" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -3600,16 +3804,16 @@
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="B140" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="C140" t="s">
         <v>6</v>
       </c>
       <c r="D140" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -3617,16 +3821,16 @@
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B141" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="C141" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D141" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -3634,16 +3838,16 @@
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="B142" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="C142" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D142" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -3651,16 +3855,16 @@
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="B143" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="C143" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D143" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -3668,16 +3872,16 @@
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="B144" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="C144" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D144" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -3685,16 +3889,16 @@
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="B145" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="C145" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D145" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -3702,16 +3906,16 @@
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="B146" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="C146" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D146" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -3719,16 +3923,16 @@
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="B147" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="C147" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="D147" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -3736,16 +3940,16 @@
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="B148" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="C148" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="D148" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -3753,16 +3957,16 @@
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="B149" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C149" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="D149" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -3770,16 +3974,16 @@
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="B150" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="C150" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="D150" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -3787,16 +3991,16 @@
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="B151" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="C151" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D151" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -3804,16 +4008,16 @@
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="B152" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="C152" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D152" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -3821,16 +4025,16 @@
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="B153" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="C153" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D153" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -3838,16 +4042,16 @@
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="B154" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="C154" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="D154" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -3855,16 +4059,16 @@
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B155" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="C155" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D155" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -3872,16 +4076,16 @@
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="B156" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="C156" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D156" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -3889,16 +4093,16 @@
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="B157" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="C157" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D157" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -3906,16 +4110,16 @@
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="B158" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="C158" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="D158" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -3923,16 +4127,16 @@
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="B159" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C159" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D159" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -3940,16 +4144,16 @@
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="B160" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="C160" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="D160" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -3957,16 +4161,16 @@
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="B161" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="C161" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D161" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -3974,16 +4178,16 @@
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="B162" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="C162" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="D162" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="E162">
         <v>1</v>
@@ -3991,16 +4195,16 @@
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="B163" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="C163" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D163" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="E163">
         <v>1</v>
@@ -4008,16 +4212,16 @@
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="B164" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="C164" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D164" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="E164">
         <v>1</v>
@@ -4025,16 +4229,16 @@
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="B165" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="C165" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D165" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="E165">
         <v>1</v>
@@ -4042,16 +4246,16 @@
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="B166" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="C166" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D166" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="E166">
         <v>1</v>
@@ -4059,16 +4263,16 @@
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="B167" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C167" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D167" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="E167">
         <v>1</v>
@@ -4076,16 +4280,16 @@
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="B168" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="C168" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="D168" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="E168">
         <v>1</v>
@@ -4093,16 +4297,16 @@
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="B169" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="C169" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D169" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -4110,16 +4314,16 @@
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="B170" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="C170" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D170" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -4127,16 +4331,16 @@
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="B171" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="C171" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D171" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -4144,16 +4348,16 @@
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="B172" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="C172" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D172" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -4161,44 +4365,50 @@
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="B173" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="C173" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D173" t="s">
-        <v>366</v>
+        <v>362</v>
+      </c>
+      <c r="E173">
+        <v>1</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="B174" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="C174" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D174" t="s">
-        <v>366</v>
+        <v>362</v>
+      </c>
+      <c r="E174">
+        <v>1</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="B175" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="C175" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="D175" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -4206,16 +4416,16 @@
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="B176" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="C176" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D176" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -4223,16 +4433,16 @@
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="B177" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="C177" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D177" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -4240,30 +4450,33 @@
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="B178" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="C178" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D178" t="s">
-        <v>379</v>
+        <v>375</v>
+      </c>
+      <c r="E178">
+        <v>1</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="B179" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="C179" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="D179" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -4271,5 +4484,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>